<commit_message>
Update Foundation public wording
</commit_message>
<xml_diff>
--- a/templates/2026-playmakers-cup-applications.xlsx
+++ b/templates/2026-playmakers-cup-applications.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="1" r:id="R77bfec05f77a4476"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review guide" sheetId="2" r:id="R583ac8e2dab246d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="1" r:id="R562e9cde469c4c40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review guide" sheetId="2" r:id="R26be4ec06d0b4d0b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4502,7 +4502,7 @@
         <x:v>Use of the award</x:v>
       </x:c>
       <x:c r="B14" s="3" t="str">
-        <x:v>No additional purchase from Playmaker Sports LLC is required. The Foundation selects the recipient and documents the charitable purpose of assistance to the athlete.</x:v>
+        <x:v>No additional purchase from Playmaker Sports is required. The Foundation selects the recipient and documents the charitable purpose of assistance to the athlete.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="56" customHeight="1">

</xml_diff>